<commit_message>
soft deletion, partial return, cancel and sales report, best selling, invoice generation
</commit_message>
<xml_diff>
--- a/sales_report.xlsx
+++ b/sales_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Order ID</t>
   </si>
@@ -53,34 +53,22 @@
     <t>Order Date</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>polyster pants</t>
-  </si>
-  <si>
-    <t>delivered</t>
+    <t>Stone Stack T-Shirt</t>
+  </si>
+  <si>
+    <t>pending</t>
   </si>
   <si>
     <t>COD</t>
   </si>
   <si>
-    <t>2024-08-08</t>
+    <t>2026-10-15</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>exclusive</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>nylon shirts</t>
+    <t>Classic T-Shirt</t>
   </si>
 </sst>
 </file>
@@ -434,248 +422,84 @@
     </row>
     <row r="2">
       <c r="A2">
+        <v>50</v>
+      </c>
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>999</v>
       </c>
       <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>99.9</v>
+      </c>
+      <c r="J2">
+        <v>104.9</v>
+      </c>
+      <c r="K2">
+        <v>1893.1</v>
+      </c>
+      <c r="L2" t="s">
         <v>15</v>
       </c>
-      <c r="H2">
-        <v>1.1904761904761905</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>1.1904761904761905</v>
-      </c>
-      <c r="K2">
-        <v>98.80952380952381</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>16</v>
-      </c>
-      <c r="M2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
       <c r="E3">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>1993</v>
+      </c>
+      <c r="L3" t="s">
         <v>15</v>
       </c>
-      <c r="H3">
-        <v>23.809523809523807</v>
-      </c>
-      <c r="I3">
-        <v>200</v>
-      </c>
-      <c r="J3">
-        <v>223.8095238095238</v>
-      </c>
-      <c r="K3">
-        <v>1776.1904761904761</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>16</v>
-      </c>
-      <c r="M3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>1000</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4">
-        <v>23.809523809523807</v>
-      </c>
-      <c r="I4">
-        <v>200</v>
-      </c>
-      <c r="J4">
-        <v>223.8095238095238</v>
-      </c>
-      <c r="K4">
-        <v>1776.1904761904761</v>
-      </c>
-      <c r="L4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>100</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5">
-        <v>1.1904761904761905</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>1.1904761904761905</v>
-      </c>
-      <c r="K5">
-        <v>98.80952380952381</v>
-      </c>
-      <c r="L5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6">
-        <v>100</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>2.380952380952381</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>2.380952380952381</v>
-      </c>
-      <c r="K6">
-        <v>197.61904761904762</v>
-      </c>
-      <c r="L6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>100</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7">
-        <v>2.380952380952381</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>2.380952380952381</v>
-      </c>
-      <c r="K7">
-        <v>197.61904761904762</v>
-      </c>
-      <c r="L7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M7" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>